<commit_message>
Corrige le binding EDQM pour Medication.form, dosage.route et quantity.unit
FRCoreValueSetEDQM était restreint à is-a #PDF mais aussi référencé par
dosage.route (classe ROA) et MedicationDispense.quantity.unit (classe
CON), ce qui ne pouvait jamais correspondre.

- Remplace FRCoreValueSetEDQM par FRCoreValueSetEDQMForm (is-a PDF,
  BDF, CDF) dédié à Medication.form.
- Ajoute FRCoreValueSetEDQMRoute (is-a ROA) pour dosage.route /
  dosageInstruction.route dans les 3 profils concernés.
- Retire le binding EDQM sur MedicationDispense.quantity.unit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 93bcf8621a6238fb384287859869d9f4a0bbd9b4
</commit_message>
<xml_diff>
--- a/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-administration.xlsx
+++ b/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-administration.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1906" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1943" uniqueCount="405">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-13T12:31:13+00:00</t>
+    <t>2026-10-15T15:33:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -718,29 +718,52 @@
     <t>MedicationAdministration.medication[x]</t>
   </si>
   <si>
+    <t>CodeableConcept
+Reference(Medication|4.0.1)</t>
+  </si>
+  <si>
+    <t>Médicament administré</t>
+  </si>
+  <si>
+    <t>Identifies the medication that was administered. This is either a link to a resource representing the details of the medication or a simple attribute carrying a code that identifies the medication from a known list of medications.</t>
+  </si>
+  <si>
+    <t>If only a code is specified, then it needs to be a code for a specific product. If more information is required, then the use of the medication resource is recommended.  For example, if you require form or lot number, then you must reference the Medication resource.</t>
+  </si>
+  <si>
+    <t>Codes identifying substance or product that can be administered.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/medication-codes|4.0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">type:$this}
+</t>
+  </si>
+  <si>
+    <t>Event.code</t>
+  </si>
+  <si>
+    <t>.participation[typeCode=CSM].role[classCode=ADMM]</t>
+  </si>
+  <si>
+    <t>FiveWs.what[x]</t>
+  </si>
+  <si>
+    <t>RXA-5-Administered Code</t>
+  </si>
+  <si>
+    <t>MedicationAdministration.medication[x]:medicationReference</t>
+  </si>
+  <si>
+    <t>medicationReference</t>
+  </si>
+  <si>
     <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-medication|2.2.0)
 </t>
   </si>
   <si>
-    <t>Médicament administré</t>
-  </si>
-  <si>
-    <t>Identifies the medication that was administered. This is either a link to a resource representing the details of the medication or a simple attribute carrying a code that identifies the medication from a known list of medications.</t>
-  </si>
-  <si>
-    <t>If only a code is specified, then it needs to be a code for a specific product. If more information is required, then the use of the medication resource is recommended.  For example, if you require form or lot number, then you must reference the Medication resource.</t>
-  </si>
-  <si>
-    <t>Event.code</t>
-  </si>
-  <si>
-    <t>.participation[typeCode=CSM].role[classCode=ADMM]</t>
-  </si>
-  <si>
-    <t>FiveWs.what[x]</t>
-  </si>
-  <si>
-    <t>RXA-5-Administered Code</t>
+    <t>What was administered</t>
   </si>
   <si>
     <t>MedicationAdministration.subject</t>
@@ -1113,7 +1136,7 @@
     <t>extensible</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-human-substance-administration-site-cisis|20260619134041</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-human-substance-administration-site-cisis|20260916095453</t>
   </si>
   <si>
     <t>.approachSiteCode</t>
@@ -1134,7 +1157,7 @@
     <t>EDQM - Standard terms / classe ROA</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-edqm|2.2.0</t>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-edqm-route|2.2.0</t>
   </si>
   <si>
     <t>.routeCode</t>
@@ -1203,10 +1226,6 @@
   </si>
   <si>
     <t>If the rate changes over time, and you want to capture this in MedicationAdministration, then each change should be captured as a distinct MedicationAdministration, with a specific MedicationAdministration.dosage.rate, and the date time when the rate change occurred. Typically, the MedicationAdministration.dosage.rate element is not used to convey an average rate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type:$this}
-</t>
   </si>
   <si>
     <t>closed</t>
@@ -1566,12 +1585,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AO51"/>
+  <dimension ref="A1:AO52"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="48.1484375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="49.765625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="44.1796875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.11328125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="17.6875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
@@ -4121,28 +4140,26 @@
         <v>79</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>79</v>
+        <v>213</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>79</v>
+        <v>230</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>79</v>
+        <v>231</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AB22" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC22" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>232</v>
+      </c>
+      <c r="AC22" s="2"/>
       <c r="AD22" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE22" t="s" s="2">
-        <v>79</v>
+        <v>138</v>
       </c>
       <c r="AF22" t="s" s="2">
         <v>225</v>
@@ -4160,16 +4177,16 @@
         <v>101</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="AM22" t="s" s="2">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="AO22" t="s" s="2">
         <v>79</v>
@@ -4177,18 +4194,20 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>234</v>
-      </c>
-      <c r="C23" s="2"/>
+        <v>225</v>
+      </c>
+      <c r="C23" t="s" s="2">
+        <v>238</v>
+      </c>
       <c r="D23" t="s" s="2">
         <v>79</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G23" t="s" s="2">
         <v>89</v>
@@ -4203,15 +4222,17 @@
         <v>90</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>237</v>
-      </c>
-      <c r="N23" s="2"/>
+        <v>228</v>
+      </c>
+      <c r="N23" t="s" s="2">
+        <v>229</v>
+      </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>79</v>
@@ -4260,7 +4281,7 @@
         <v>79</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>89</v>
@@ -4275,16 +4296,16 @@
         <v>101</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="AO23" t="s" s="2">
         <v>79</v>
@@ -4292,10 +4313,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4303,7 +4324,7 @@
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G24" t="s" s="2">
         <v>89</v>
@@ -4315,16 +4336,16 @@
         <v>79</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="K24" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="L24" t="s" s="2">
         <v>243</v>
       </c>
-      <c r="L24" t="s" s="2">
+      <c r="M24" t="s" s="2">
         <v>244</v>
-      </c>
-      <c r="M24" t="s" s="2">
-        <v>245</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -4375,10 +4396,10 @@
         <v>79</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="AG24" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AH24" t="s" s="2">
         <v>89</v>
@@ -4390,16 +4411,16 @@
         <v>101</v>
       </c>
       <c r="AK24" t="s" s="2">
+        <v>245</v>
+      </c>
+      <c r="AL24" t="s" s="2">
         <v>246</v>
       </c>
-      <c r="AL24" t="s" s="2">
+      <c r="AM24" t="s" s="2">
         <v>247</v>
       </c>
-      <c r="AM24" t="s" s="2">
+      <c r="AN24" t="s" s="2">
         <v>248</v>
-      </c>
-      <c r="AN24" t="s" s="2">
-        <v>249</v>
       </c>
       <c r="AO24" t="s" s="2">
         <v>79</v>
@@ -4407,10 +4428,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4421,7 +4442,7 @@
         <v>80</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>79</v>
@@ -4433,13 +4454,13 @@
         <v>79</v>
       </c>
       <c r="K25" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="L25" t="s" s="2">
         <v>251</v>
       </c>
-      <c r="L25" t="s" s="2">
+      <c r="M25" t="s" s="2">
         <v>252</v>
-      </c>
-      <c r="M25" t="s" s="2">
-        <v>253</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -4490,13 +4511,13 @@
         <v>79</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>79</v>
@@ -4505,16 +4526,16 @@
         <v>101</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>79</v>
+        <v>253</v>
       </c>
       <c r="AL25" t="s" s="2">
         <v>254</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="AN25" t="s" s="2">
-        <v>79</v>
+        <v>256</v>
       </c>
       <c r="AO25" t="s" s="2">
         <v>79</v>
@@ -4522,10 +4543,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4533,10 +4554,10 @@
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="H26" t="s" s="2">
         <v>79</v>
@@ -4545,16 +4566,16 @@
         <v>79</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
@@ -4605,13 +4626,13 @@
         <v>79</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="AG26" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AH26" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="AI26" t="s" s="2">
         <v>79</v>
@@ -4620,16 +4641,16 @@
         <v>101</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>259</v>
+        <v>79</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="AN26" t="s" s="2">
-        <v>262</v>
+        <v>79</v>
       </c>
       <c r="AO26" t="s" s="2">
         <v>79</v>
@@ -4637,10 +4658,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4648,10 +4669,10 @@
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>79</v>
@@ -4663,13 +4684,13 @@
         <v>90</v>
       </c>
       <c r="K27" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="L27" t="s" s="2">
         <v>264</v>
       </c>
-      <c r="L27" t="s" s="2">
+      <c r="M27" t="s" s="2">
         <v>265</v>
-      </c>
-      <c r="M27" t="s" s="2">
-        <v>266</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4720,13 +4741,13 @@
         <v>79</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AG27" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>79</v>
@@ -4735,16 +4756,16 @@
         <v>101</v>
       </c>
       <c r="AK27" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="AL27" t="s" s="2">
         <v>267</v>
       </c>
-      <c r="AL27" t="s" s="2">
+      <c r="AM27" t="s" s="2">
         <v>268</v>
       </c>
-      <c r="AM27" t="s" s="2">
+      <c r="AN27" t="s" s="2">
         <v>269</v>
-      </c>
-      <c r="AN27" t="s" s="2">
-        <v>270</v>
       </c>
       <c r="AO27" t="s" s="2">
         <v>79</v>
@@ -4752,10 +4773,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4766,7 +4787,7 @@
         <v>80</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>79</v>
@@ -4775,16 +4796,16 @@
         <v>79</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>150</v>
+        <v>271</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>151</v>
+        <v>272</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>152</v>
+        <v>273</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -4835,31 +4856,31 @@
         <v>79</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>153</v>
+        <v>270</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>79</v>
+        <v>274</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>154</v>
+        <v>275</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>79</v>
+        <v>276</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>79</v>
+        <v>277</v>
       </c>
       <c r="AO28" t="s" s="2">
         <v>79</v>
@@ -4867,21 +4888,21 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>173</v>
+        <v>79</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>79</v>
@@ -4893,17 +4914,15 @@
         <v>79</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>273</v>
+        <v>151</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>274</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>176</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>79</v>
@@ -4952,19 +4971,19 @@
         <v>79</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>140</v>
+        <v>79</v>
       </c>
       <c r="AK29" t="s" s="2">
         <v>79</v>
@@ -4984,14 +5003,14 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>276</v>
+        <v>173</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -5004,26 +5023,24 @@
         <v>79</v>
       </c>
       <c r="I30" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="K30" t="s" s="2">
         <v>134</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="N30" t="s" s="2">
         <v>176</v>
       </c>
-      <c r="O30" t="s" s="2">
-        <v>177</v>
-      </c>
+      <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>79</v>
       </c>
@@ -5071,7 +5088,7 @@
         <v>79</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>279</v>
+        <v>158</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>80</v>
@@ -5089,7 +5106,7 @@
         <v>79</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>79</v>
@@ -5103,42 +5120,46 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>79</v>
+        <v>283</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I31" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>210</v>
+        <v>134</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>282</v>
-      </c>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
+        <v>285</v>
+      </c>
+      <c r="N31" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="O31" t="s" s="2">
+        <v>177</v>
+      </c>
       <c r="P31" t="s" s="2">
         <v>79</v>
       </c>
@@ -5162,13 +5183,13 @@
         <v>79</v>
       </c>
       <c r="X31" t="s" s="2">
-        <v>213</v>
+        <v>79</v>
       </c>
       <c r="Y31" t="s" s="2">
-        <v>283</v>
+        <v>79</v>
       </c>
       <c r="Z31" t="s" s="2">
-        <v>284</v>
+        <v>79</v>
       </c>
       <c r="AA31" t="s" s="2">
         <v>79</v>
@@ -5186,25 +5207,25 @@
         <v>79</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>285</v>
+        <v>79</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>286</v>
+        <v>132</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>79</v>
@@ -5229,7 +5250,7 @@
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="G32" t="s" s="2">
         <v>89</v>
@@ -5241,16 +5262,16 @@
         <v>79</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="K32" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="L32" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="L32" t="s" s="2">
+      <c r="M32" t="s" s="2">
         <v>289</v>
-      </c>
-      <c r="M32" t="s" s="2">
-        <v>290</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -5277,13 +5298,13 @@
         <v>79</v>
       </c>
       <c r="X32" t="s" s="2">
-        <v>79</v>
+        <v>213</v>
       </c>
       <c r="Y32" t="s" s="2">
-        <v>79</v>
+        <v>290</v>
       </c>
       <c r="Z32" t="s" s="2">
-        <v>79</v>
+        <v>291</v>
       </c>
       <c r="AA32" t="s" s="2">
         <v>79</v>
@@ -5304,7 +5325,7 @@
         <v>287</v>
       </c>
       <c r="AG32" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AH32" t="s" s="2">
         <v>89</v>
@@ -5316,10 +5337,10 @@
         <v>101</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>79</v>
@@ -5333,10 +5354,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5344,10 +5365,10 @@
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>79</v>
@@ -5356,16 +5377,16 @@
         <v>79</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>210</v>
+        <v>295</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -5392,13 +5413,13 @@
         <v>79</v>
       </c>
       <c r="X33" t="s" s="2">
-        <v>213</v>
+        <v>79</v>
       </c>
       <c r="Y33" t="s" s="2">
-        <v>296</v>
+        <v>79</v>
       </c>
       <c r="Z33" t="s" s="2">
-        <v>297</v>
+        <v>79</v>
       </c>
       <c r="AA33" t="s" s="2">
         <v>79</v>
@@ -5416,13 +5437,13 @@
         <v>79</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="AG33" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>79</v>
@@ -5440,7 +5461,7 @@
         <v>79</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>300</v>
+        <v>79</v>
       </c>
       <c r="AO33" t="s" s="2">
         <v>79</v>
@@ -5448,10 +5469,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5474,17 +5495,15 @@
         <v>79</v>
       </c>
       <c r="K34" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="L34" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="M34" t="s" s="2">
         <v>302</v>
       </c>
-      <c r="L34" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="M34" t="s" s="2">
-        <v>304</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>305</v>
-      </c>
+      <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>79</v>
@@ -5509,13 +5528,13 @@
         <v>79</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>79</v>
+        <v>213</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>79</v>
+        <v>303</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>79</v>
+        <v>304</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>79</v>
@@ -5533,7 +5552,7 @@
         <v>79</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>80</v>
@@ -5548,27 +5567,27 @@
         <v>101</v>
       </c>
       <c r="AK34" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="AL34" t="s" s="2">
         <v>306</v>
       </c>
-      <c r="AL34" t="s" s="2">
+      <c r="AM34" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AN34" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="AM34" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="AN34" t="s" s="2">
-        <v>79</v>
-      </c>
       <c r="AO34" t="s" s="2">
-        <v>309</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5579,7 +5598,7 @@
         <v>80</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>79</v>
@@ -5591,16 +5610,16 @@
         <v>79</v>
       </c>
       <c r="K35" t="s" s="2">
+        <v>309</v>
+      </c>
+      <c r="L35" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="M35" t="s" s="2">
         <v>311</v>
       </c>
-      <c r="L35" t="s" s="2">
+      <c r="N35" t="s" s="2">
         <v>312</v>
-      </c>
-      <c r="M35" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>314</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5650,13 +5669,13 @@
         <v>79</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>79</v>
@@ -5665,27 +5684,27 @@
         <v>101</v>
       </c>
       <c r="AK35" t="s" s="2">
+        <v>313</v>
+      </c>
+      <c r="AL35" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="AM35" t="s" s="2">
         <v>315</v>
       </c>
-      <c r="AL35" t="s" s="2">
+      <c r="AN35" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO35" t="s" s="2">
         <v>316</v>
-      </c>
-      <c r="AM35" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN35" t="s" s="2">
-        <v>317</v>
-      </c>
-      <c r="AO35" t="s" s="2">
-        <v>79</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5696,7 +5715,7 @@
         <v>80</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>79</v>
@@ -5708,15 +5727,17 @@
         <v>79</v>
       </c>
       <c r="K36" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="L36" t="s" s="2">
         <v>319</v>
       </c>
-      <c r="L36" t="s" s="2">
+      <c r="M36" t="s" s="2">
         <v>320</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="N36" t="s" s="2">
         <v>321</v>
       </c>
-      <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>79</v>
@@ -5765,13 +5786,13 @@
         <v>79</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>79</v>
@@ -5780,16 +5801,16 @@
         <v>101</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>79</v>
+        <v>322</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="AM36" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="AO36" t="s" s="2">
         <v>79</v>
@@ -5797,10 +5818,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5823,13 +5844,13 @@
         <v>79</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -5880,7 +5901,7 @@
         <v>79</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>80</v>
@@ -5895,7 +5916,7 @@
         <v>101</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>328</v>
+        <v>79</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>329</v>
@@ -5904,7 +5925,7 @@
         <v>79</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>79</v>
+        <v>330</v>
       </c>
       <c r="AO37" t="s" s="2">
         <v>79</v>
@@ -5912,10 +5933,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5926,7 +5947,7 @@
         <v>80</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>79</v>
@@ -5938,13 +5959,13 @@
         <v>79</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>264</v>
+        <v>332</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5995,25 +6016,25 @@
         <v>79</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>333</v>
+        <v>101</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>79</v>
+        <v>335</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="AM38" t="s" s="2">
         <v>79</v>
@@ -6027,10 +6048,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6053,13 +6074,13 @@
         <v>79</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>150</v>
+        <v>271</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>151</v>
+        <v>338</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>152</v>
+        <v>339</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -6110,7 +6131,7 @@
         <v>79</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>153</v>
+        <v>337</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>80</v>
@@ -6122,13 +6143,13 @@
         <v>79</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>79</v>
+        <v>340</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>154</v>
+        <v>341</v>
       </c>
       <c r="AM39" t="s" s="2">
         <v>79</v>
@@ -6142,10 +6163,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6156,7 +6177,7 @@
         <v>80</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>79</v>
@@ -6168,13 +6189,13 @@
         <v>79</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -6213,35 +6234,37 @@
         <v>79</v>
       </c>
       <c r="AB40" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="AC40" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="AC40" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="AD40" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE40" t="s" s="2">
-        <v>138</v>
+        <v>79</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>140</v>
+        <v>79</v>
       </c>
       <c r="AK40" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>79</v>
+        <v>154</v>
       </c>
       <c r="AM40" t="s" s="2">
         <v>79</v>
@@ -6255,14 +6278,12 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>336</v>
-      </c>
-      <c r="C41" t="s" s="2">
-        <v>338</v>
-      </c>
+        <v>343</v>
+      </c>
+      <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
         <v>79</v>
       </c>
@@ -6283,13 +6304,13 @@
         <v>79</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>339</v>
+        <v>134</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>340</v>
+        <v>135</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>341</v>
+        <v>136</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6328,16 +6349,14 @@
         <v>79</v>
       </c>
       <c r="AB41" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC41" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="AC41" s="2"/>
       <c r="AD41" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE41" t="s" s="2">
-        <v>79</v>
+        <v>138</v>
       </c>
       <c r="AF41" t="s" s="2">
         <v>158</v>
@@ -6349,7 +6368,7 @@
         <v>81</v>
       </c>
       <c r="AI41" t="s" s="2">
-        <v>147</v>
+        <v>79</v>
       </c>
       <c r="AJ41" t="s" s="2">
         <v>140</v>
@@ -6372,14 +6391,16 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>342</v>
-      </c>
-      <c r="C42" s="2"/>
+        <v>343</v>
+      </c>
+      <c r="C42" t="s" s="2">
+        <v>345</v>
+      </c>
       <c r="D42" t="s" s="2">
-        <v>276</v>
+        <v>79</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -6392,26 +6413,22 @@
         <v>79</v>
       </c>
       <c r="I42" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>134</v>
+        <v>346</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>277</v>
+        <v>347</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>278</v>
-      </c>
-      <c r="N42" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="O42" t="s" s="2">
-        <v>177</v>
-      </c>
+        <v>348</v>
+      </c>
+      <c r="N42" s="2"/>
+      <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
         <v>79</v>
       </c>
@@ -6459,7 +6476,7 @@
         <v>79</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>279</v>
+        <v>158</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>80</v>
@@ -6468,7 +6485,7 @@
         <v>81</v>
       </c>
       <c r="AI42" t="s" s="2">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="AJ42" t="s" s="2">
         <v>140</v>
@@ -6477,7 +6494,7 @@
         <v>79</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>132</v>
+        <v>79</v>
       </c>
       <c r="AM42" t="s" s="2">
         <v>79</v>
@@ -6491,42 +6508,46 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>79</v>
+        <v>283</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I43" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>344</v>
+        <v>284</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>345</v>
-      </c>
-      <c r="N43" s="2"/>
-      <c r="O43" s="2"/>
+        <v>285</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="O43" t="s" s="2">
+        <v>177</v>
+      </c>
       <c r="P43" t="s" s="2">
         <v>79</v>
       </c>
@@ -6574,25 +6595,25 @@
         <v>79</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>343</v>
+        <v>286</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>346</v>
+        <v>132</v>
       </c>
       <c r="AM43" t="s" s="2">
         <v>79</v>
@@ -6606,10 +6627,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6632,17 +6653,15 @@
         <v>79</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>210</v>
+        <v>150</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>349</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>350</v>
-      </c>
+        <v>352</v>
+      </c>
+      <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>79</v>
@@ -6667,11 +6686,13 @@
         <v>79</v>
       </c>
       <c r="X44" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="Y44" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="Y44" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="Z44" t="s" s="2">
-        <v>352</v>
+        <v>79</v>
       </c>
       <c r="AA44" t="s" s="2">
         <v>79</v>
@@ -6689,7 +6710,7 @@
         <v>79</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>80</v>
@@ -6713,7 +6734,7 @@
         <v>79</v>
       </c>
       <c r="AN44" t="s" s="2">
-        <v>354</v>
+        <v>79</v>
       </c>
       <c r="AO44" t="s" s="2">
         <v>79</v>
@@ -6721,10 +6742,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6750,12 +6771,14 @@
         <v>210</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>356</v>
       </c>
-      <c r="M45" t="s" s="2">
+      <c r="N45" t="s" s="2">
         <v>357</v>
       </c>
-      <c r="N45" s="2"/>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>79</v>
@@ -6780,11 +6803,9 @@
         <v>79</v>
       </c>
       <c r="X45" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="Y45" t="s" s="2">
         <v>358</v>
       </c>
+      <c r="Y45" s="2"/>
       <c r="Z45" t="s" s="2">
         <v>359</v>
       </c>
@@ -6804,7 +6825,7 @@
         <v>79</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>80</v>
@@ -6870,9 +6891,7 @@
       <c r="M46" t="s" s="2">
         <v>364</v>
       </c>
-      <c r="N46" t="s" s="2">
-        <v>365</v>
-      </c>
+      <c r="N46" s="2"/>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>79</v>
@@ -6897,13 +6916,13 @@
         <v>79</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>213</v>
+        <v>358</v>
       </c>
       <c r="Y46" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="Z46" t="s" s="2">
         <v>366</v>
-      </c>
-      <c r="Z46" t="s" s="2">
-        <v>367</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>79</v>
@@ -6939,13 +6958,13 @@
         <v>79</v>
       </c>
       <c r="AL46" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="AM46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AN46" t="s" s="2">
         <v>368</v>
-      </c>
-      <c r="AM46" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AN46" t="s" s="2">
-        <v>369</v>
       </c>
       <c r="AO46" t="s" s="2">
         <v>79</v>
@@ -6953,10 +6972,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6979,16 +6998,16 @@
         <v>79</v>
       </c>
       <c r="K47" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="L47" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="M47" t="s" s="2">
         <v>371</v>
       </c>
-      <c r="L47" t="s" s="2">
+      <c r="N47" t="s" s="2">
         <v>372</v>
-      </c>
-      <c r="M47" t="s" s="2">
-        <v>373</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>374</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -7014,13 +7033,13 @@
         <v>79</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>79</v>
+        <v>213</v>
       </c>
       <c r="Y47" t="s" s="2">
-        <v>79</v>
+        <v>373</v>
       </c>
       <c r="Z47" t="s" s="2">
-        <v>79</v>
+        <v>374</v>
       </c>
       <c r="AA47" t="s" s="2">
         <v>79</v>
@@ -7038,7 +7057,7 @@
         <v>79</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>80</v>
@@ -7143,14 +7162,16 @@
         <v>79</v>
       </c>
       <c r="AB48" t="s" s="2">
-        <v>382</v>
-      </c>
-      <c r="AC48" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="AC48" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="AD48" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE48" t="s" s="2">
-        <v>383</v>
+        <v>79</v>
       </c>
       <c r="AF48" t="s" s="2">
         <v>377</v>
@@ -7171,13 +7192,13 @@
         <v>79</v>
       </c>
       <c r="AL48" t="s" s="2">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="AM48" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN48" t="s" s="2">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="AO48" t="s" s="2">
         <v>79</v>
@@ -7185,14 +7206,12 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>377</v>
-      </c>
-      <c r="C49" t="s" s="2">
-        <v>387</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
         <v>79</v>
       </c>
@@ -7213,16 +7232,16 @@
         <v>79</v>
       </c>
       <c r="K49" t="s" s="2">
+        <v>385</v>
+      </c>
+      <c r="L49" t="s" s="2">
+        <v>386</v>
+      </c>
+      <c r="M49" t="s" s="2">
+        <v>387</v>
+      </c>
+      <c r="N49" t="s" s="2">
         <v>388</v>
-      </c>
-      <c r="L49" t="s" s="2">
-        <v>389</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>380</v>
-      </c>
-      <c r="N49" t="s" s="2">
-        <v>381</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
@@ -7260,19 +7279,17 @@
         <v>79</v>
       </c>
       <c r="AB49" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>232</v>
+      </c>
+      <c r="AC49" s="2"/>
       <c r="AD49" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE49" t="s" s="2">
-        <v>79</v>
+        <v>389</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>80</v>
@@ -7290,13 +7307,13 @@
         <v>79</v>
       </c>
       <c r="AL49" t="s" s="2">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="AM49" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN49" t="s" s="2">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="AO49" t="s" s="2">
         <v>79</v>
@@ -7304,13 +7321,13 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="C50" t="s" s="2">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="D50" t="s" s="2">
         <v>79</v>
@@ -7332,16 +7349,16 @@
         <v>79</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>371</v>
+        <v>394</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="N50" t="s" s="2">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
@@ -7391,7 +7408,7 @@
         <v>79</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>80</v>
@@ -7409,13 +7426,13 @@
         <v>79</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="AM50" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN50" t="s" s="2">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="AO50" t="s" s="2">
         <v>79</v>
@@ -7423,12 +7440,14 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>393</v>
-      </c>
-      <c r="C51" s="2"/>
+        <v>384</v>
+      </c>
+      <c r="C51" t="s" s="2">
+        <v>397</v>
+      </c>
       <c r="D51" t="s" s="2">
         <v>79</v>
       </c>
@@ -7437,7 +7456,7 @@
         <v>80</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="H51" t="s" s="2">
         <v>79</v>
@@ -7449,16 +7468,16 @@
         <v>79</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>394</v>
+        <v>378</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="N51" t="s" s="2">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
@@ -7508,13 +7527,13 @@
         <v>79</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH51" t="s" s="2">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="AI51" t="s" s="2">
         <v>79</v>
@@ -7526,15 +7545,132 @@
         <v>79</v>
       </c>
       <c r="AL51" t="s" s="2">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="AM51" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AN51" t="s" s="2">
-        <v>79</v>
+        <v>391</v>
       </c>
       <c r="AO51" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="2">
+        <v>399</v>
+      </c>
+      <c r="B52" t="s" s="2">
+        <v>399</v>
+      </c>
+      <c r="C52" s="2"/>
+      <c r="D52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E52" s="2"/>
+      <c r="F52" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="K52" t="s" s="2">
+        <v>400</v>
+      </c>
+      <c r="L52" t="s" s="2">
+        <v>401</v>
+      </c>
+      <c r="M52" t="s" s="2">
+        <v>402</v>
+      </c>
+      <c r="N52" t="s" s="2">
+        <v>403</v>
+      </c>
+      <c r="O52" s="2"/>
+      <c r="P52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q52" s="2"/>
+      <c r="R52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF52" t="s" s="2">
+        <v>399</v>
+      </c>
+      <c r="AG52" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ52" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="AK52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AL52" t="s" s="2">
+        <v>404</v>
+      </c>
+      <c r="AM52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AN52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AO52" t="s" s="2">
         <v>79</v>
       </c>
     </row>

</xml_diff>